<commit_message>
Add reseller-direct valuation with certified data-wipe deduction
Rework the used-value estimate for a direct wholesale sale to a reseller:
net offer = retail resale x ~50% wholesale factor, minus a certified
NIST 800-88 data-sanitization allowance (drives retained). Adds a
reseller-direct sheet, keeps the retail resale reference, and updates
methodology and README.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QtXzSQeVtnWoqeQMAXgubX
</commit_message>
<xml_diff>
--- a/renew-it-resources/2026-07-07_Inventory/HPE_Nimble_Used_Price_Estimate_2026-07-07.xlsx
+++ b/renew-it-resources/2026-07-07_Inventory/HPE_Nimble_Used_Price_Estimate_2026-07-07.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Used Price Estimate" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sources &amp; Methodology" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Reseller-Direct Offer (Wiped)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Retail Resale (Reference)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sources &amp; Methodology" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50,7 +51,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +61,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -99,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -112,7 +123,16 @@
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -121,7 +141,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -488,46 +515,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HPE Nimble Storage — Estimated Used / Secondary-Market Values</t>
+          <t>HPE Nimble Storage — Estimated Reseller-Direct Offer (Sold to Reseller, Certified Data Wipe Included)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Renew IT Resources  |  Inventory date: 2026-07-07  |  All arrays HW EOS 7/31/2028 (still HPE-supportable, sustains resale)</t>
+          <t>Renew IT Resources  |  2026-07-07  |  Direct-to-reseller wholesale sale. Reseller performs certified NIST 800-88 data sanitization (drives retained) with Certificate of Destruction.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Estimates are fair-market used values for the base array (dual controller). USD. Exclude shipping, tax, support renewal, and installed data. Ranges reflect condition, config &amp; network-adapter variance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Net Offer = (Retail resale value × reseller wholesale factor ~50%) − certified data-wipe allowance. USD. Excludes shipping, tax, and active HPE support renewal. All arrays HW EOS 7/31/2028 (still supportable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>#</t>
@@ -535,12 +564,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Array S/N</t>
+          <t>S/N</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Datacenter</t>
+          <t>DC</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -555,46 +584,62 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Shelves</t>
+          <t>HDD (TB)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>HDD Raw (TB)</t>
+          <t>SSD (TB)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>SSD Raw (TB)</t>
+          <t>Est. Drives</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Host Interface</t>
+          <t>Retail Resale
+(reference)</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Est. Low (USD)</t>
+          <t>Reseller Gross
+@ ~50%</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Est. Point (USD)</t>
+          <t>Data-Wipe
+Allowance</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Est. High (USD)</t>
+          <t>Net Offer
+Low</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Pricing Basis</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
+          <t>Net Offer
+Point</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Net Offer
+High</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>1</v>
       </c>
@@ -620,36 +665,42 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>126</v>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>11.52</t>
+        </is>
       </c>
       <c r="H6" s="4" t="n">
-        <v>11.52</v>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K6" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="I6" s="5" t="n">
         <v>16875</v>
       </c>
-      <c r="L6" s="5" t="n">
-        <v>18000</v>
-      </c>
-      <c r="M6" s="7" t="inlineStr">
-        <is>
-          <t>Exact-match refurb listing: HF40 126TB HDD + 11.52TB SSD sells at $16,875.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
+      <c r="J6" s="6" t="n">
+        <v>8400</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>216</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>6900</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>8200</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <v>9600</v>
+      </c>
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t>~21 HDD + 6 SSD; no shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>2</v>
       </c>
@@ -673,38 +724,44 @@
           <t>All Flash</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>1</v>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>253</t>
         </is>
       </c>
       <c r="H7" s="4" t="n">
-        <v>253</v>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>4× Dual 10GbE SFP+</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="n">
-        <v>42000</v>
-      </c>
-      <c r="K7" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="I7" s="5" t="n">
         <v>47000</v>
       </c>
-      <c r="L7" s="5" t="n">
-        <v>52000</v>
-      </c>
-      <c r="M7" s="7" t="inlineStr">
-        <is>
-          <t>AF60 184TB base ~$34,950; +~69TB SSD &amp; expansion shelf. Largest AF60 here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
+      <c r="J7" s="6" t="n">
+        <v>23500</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>384</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>19400</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>23100</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>26900</v>
+      </c>
+      <c r="O7" s="10" t="inlineStr">
+        <is>
+          <t>Largest AF60; 1 expansion shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>3</v>
       </c>
@@ -728,38 +785,44 @@
           <t>All Flash</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n">
-        <v>1</v>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>184</t>
         </is>
       </c>
       <c r="H8" s="4" t="n">
-        <v>184</v>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>4× Dual 10GbE SFP+</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>33000</v>
-      </c>
-      <c r="K8" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="I8" s="5" t="n">
         <v>37000</v>
       </c>
-      <c r="L8" s="5" t="n">
-        <v>41000</v>
-      </c>
-      <c r="M8" s="7" t="inlineStr">
-        <is>
-          <t>AF60 184TB base ~$34,950 + 1 expansion shelf.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
+      <c r="J8" s="6" t="n">
+        <v>18500</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>384</v>
+      </c>
+      <c r="L8" s="8" t="n">
+        <v>15200</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>18100</v>
+      </c>
+      <c r="N8" s="8" t="n">
+        <v>21100</v>
+      </c>
+      <c r="O8" s="10" t="inlineStr">
+        <is>
+          <t>48×3.84TB SSD; 1 shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>4</v>
       </c>
@@ -783,38 +846,44 @@
           <t>All Flash</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>0</v>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>184</t>
         </is>
       </c>
       <c r="H9" s="4" t="n">
-        <v>184</v>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>4× Dual 10GbE SFP+; 1× Dual 10GBaseT</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>31000</v>
-      </c>
-      <c r="K9" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="I9" s="5" t="n">
         <v>34950</v>
       </c>
-      <c r="L9" s="5" t="n">
-        <v>38000</v>
-      </c>
-      <c r="M9" s="7" t="inlineStr">
-        <is>
-          <t>Exact-match: AF60 184TB (48×3.84TB) used listed $34,950.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
+      <c r="J9" s="6" t="n">
+        <v>17500</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>192</v>
+      </c>
+      <c r="L9" s="8" t="n">
+        <v>14500</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>17300</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>20100</v>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>24×7.68TB SSD; no shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>5</v>
       </c>
@@ -838,36 +907,44 @@
           <t>Hybrid Flash</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>294</v>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>294</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>34.6</t>
+        </is>
       </c>
       <c r="H10" s="4" t="n">
-        <v>34.6</v>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>3× Dual 10GbE SFP+</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="n">
-        <v>26000</v>
-      </c>
-      <c r="K10" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="I10" s="5" t="n">
         <v>30000</v>
       </c>
-      <c r="L10" s="5" t="n">
-        <v>34000</v>
-      </c>
-      <c r="M10" s="7" t="inlineStr">
-        <is>
-          <t>HF60 210TB used ~$23,995; larger 294TB HDD + 34.6TB cache + shelf.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
+      <c r="J10" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>384</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>12200</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>14600</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>17000</v>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>~42 HDD + 6 SSD; 1 shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>6</v>
       </c>
@@ -891,38 +968,44 @@
           <t>All Flash</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>0</v>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>184</t>
         </is>
       </c>
       <c r="H11" s="4" t="n">
-        <v>184</v>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>4× Dual 10GbE SFP+</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>55000</v>
-      </c>
-      <c r="K11" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="I11" s="5" t="n">
         <v>65000</v>
       </c>
-      <c r="L11" s="5" t="n">
-        <v>79000</v>
-      </c>
-      <c r="M11" s="7" t="inlineStr">
-        <is>
-          <t>AF80 184TB used listed $79,500 or best offer; flagship controller.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
+      <c r="J11" s="6" t="n">
+        <v>32500</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>192</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>27100</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>32300</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>37500</v>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>Flagship AF80; no shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>7</v>
       </c>
@@ -946,38 +1029,44 @@
           <t>All Flash</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>0</v>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>46.1</t>
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>2× Dual 10GbE SFP+</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="n">
-        <v>9000</v>
-      </c>
-      <c r="K12" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="I12" s="5" t="n">
         <v>12000</v>
       </c>
-      <c r="L12" s="5" t="n">
-        <v>14000</v>
-      </c>
-      <c r="M12" s="7" t="inlineStr">
-        <is>
-          <t>AF40 46TB new ~$19,995; used ~55-65% of new.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
+      <c r="J12" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>192</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>4800</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>5800</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>6800</v>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>24×1.92TB SSD; no shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>8</v>
       </c>
@@ -1001,36 +1090,44 @@
           <t>Hybrid Flash</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>168</v>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>168</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>32.6</t>
+        </is>
       </c>
       <c r="H13" s="4" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>2× Dual 10GbE SFP+</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="n">
-        <v>19000</v>
-      </c>
-      <c r="K13" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="I13" s="5" t="n">
         <v>23000</v>
       </c>
-      <c r="L13" s="5" t="n">
-        <v>27000</v>
-      </c>
-      <c r="M13" s="7" t="inlineStr">
-        <is>
-          <t>HF60 mid config; scaled below 294TB unit, includes 1 shelf.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
+      <c r="J13" s="6" t="n">
+        <v>11500</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>384</v>
+      </c>
+      <c r="L13" s="8" t="n">
+        <v>9300</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>11100</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <v>13000</v>
+      </c>
+      <c r="O13" s="10" t="inlineStr">
+        <is>
+          <t>~42 HDD + 6 SSD; 1 shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>9</v>
       </c>
@@ -1054,49 +1151,66 @@
           <t>Hybrid Flash</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>126</v>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>17.3</t>
+        </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>17.3</v>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>3× Dual 10GbE SFP+</t>
-        </is>
-      </c>
-      <c r="J14" s="5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K14" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I14" s="5" t="n">
         <v>18000</v>
       </c>
-      <c r="L14" s="5" t="n">
-        <v>21000</v>
-      </c>
-      <c r="M14" s="7" t="inlineStr">
-        <is>
-          <t>HF60 base, 126TB HDD + 17.3TB cache, no expansion shelf.</t>
+      <c r="J14" s="6" t="n">
+        <v>9000</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="L14" s="8" t="n">
+        <v>7300</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>8800</v>
+      </c>
+      <c r="N14" s="8" t="n">
+        <v>10200</v>
+      </c>
+      <c r="O14" s="10" t="inlineStr">
+        <is>
+          <t>~21 HDD + 9 SSD; no shelf</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="I15" s="8" t="inlineStr">
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTAL</t>
         </is>
       </c>
-      <c r="J15" s="9" t="n">
-        <v>245000</v>
-      </c>
-      <c r="K15" s="9" t="n">
+      <c r="I15" s="12" t="n">
         <v>283825</v>
       </c>
-      <c r="L15" s="9" t="n">
-        <v>324000</v>
+      <c r="J15" s="13" t="n">
+        <v>141900</v>
+      </c>
+      <c r="K15" s="14" t="n">
+        <v>2568</v>
+      </c>
+      <c r="L15" s="15" t="n">
+        <v>116700</v>
+      </c>
+      <c r="M15" s="15" t="n">
+        <v>139300</v>
+      </c>
+      <c r="N15" s="15" t="n">
+        <v>162200</v>
       </c>
     </row>
   </sheetData>
@@ -1110,15 +1224,493 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="115" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Retail / Secondary-Market Resale Values — Reference Basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>What an end buyer pays a reseller. The reseller-direct offer (Sheet 1) is derived from these figures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>S/N</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>HDD (TB)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>SSD (TB)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Retail Low</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Retail Point</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Retail High</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>0862</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>HF40</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>126</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>16875</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>18000</v>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>Exact-match refurb listing $16,875</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>4469</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>AF60</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>All-Flash</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>253</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>42000</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>47000</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>52000</v>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>AF60 184TB $34,950 base + capacity/shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>7343</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>AF60</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>All-Flash</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>184</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>33000</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>37000</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>41000</v>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>AF60 184TB $34,950 + 1 shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>8949</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>AF60</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>All-Flash</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>184</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>31000</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>34950</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>38000</v>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>Exact-match AF60 184TB $34,950</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>4349</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>HF60</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>294</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>26000</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>34000</v>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>HF60 210TB $23,995 scaled up + shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>1130</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>AF80</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>All-Flash</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>184</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>55000</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>65000</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>79000</v>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>AF80 184TB $79,500 or best offer</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>1813</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>AF40</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>All-Flash</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>9000</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>12000</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>14000</v>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>AF40 46TB new $19,995; used-scaled</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>1843</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>HF60</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>168</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>19000</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>23000</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>27000</v>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>HF60 mid config + shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>8863</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>HF60</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>126</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>18000</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>21000</v>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>HF60 base, no shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>245000</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>283825</v>
+      </c>
+      <c r="I14" s="15" t="n">
+        <v>324000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>Sources &amp; Methodology</t>
         </is>
       </c>
@@ -1127,186 +1719,272 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>METHODOLOGY</t>
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>SCENARIO — DIRECT SALE TO RESELLER, CERTIFIED DATA WIPE INCLUDED</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>• 'Used account' pricing = fair-market secondary/refurbished value for the base dual-controller array as configured.</t>
+          <t>• Seller sells the arrays wholesale directly to a reseller/ITAD firm (not to an end user), accepting a price cut for speed &amp; certainty.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>• Anchored to live refurbished-dealer and eBay listings (July 2026), then scaled by raw capacity, controller class (AF40&lt;AF60&lt;AF80; HF40&lt;HF60) and expansion shelves.</t>
+          <t>• Reseller provides certified data sanitization to NIST 800-88 'Purge' (crypto-erase / secure-erase) WITH a Certificate of Destruction.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>• Point = most-likely transaction price; Low/High bracket condition, warranty, and network-adapter variance.</t>
+          <t>• Drives are sanitized and RETAINED in the arrays (not physically shredded), so flash/HDD value is preserved and resold with the unit.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>• All arrays share HW End-of-Support 7/31/2028 — still supportable, which preserves resale demand today.</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>• Excludes: shipping, tax, active HPE support/InfoSight renewal, professional services, and any resident data.</t>
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>HOW EACH NET OFFER IS BUILT</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>• Net Offer = (Retail resale value × reseller wholesale factor) − certified data-wipe allowance.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>MARKET ANCHORS USED</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>• Reseller wholesale factor: Point 50%, Low 42%, High 58% of retail resale. Reflects reseller margin for refurb, warranty, holding &amp; resale risk.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>• HF40 126TB HDD + 11.52TB SSD refurb — $16,875 (Enterasource) — exact match to array #1.</t>
+          <t>• Data-wipe allowance: ~$8 per drive (certified NIST 800-88 sanitization + certificate), deducted from the reseller's gross offer.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>• HF60 210TB HDD + 23.04TB cache used — $23,995 (eBay, Core 4 Solutions).</t>
+          <t>• Retail resale values (Sheet 2) are anchored to live July-2026 refurbished-dealer and eBay listings, then scaled by capacity/controller/shelves.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>• AF60 184TB (48×3.84TB SSD) used — $34,950 (eBay) — matches arrays #3/#4.</t>
+          <t>• All arrays share HW End-of-Support 7/31/2028 — still supportable, which sustains reseller demand and buy prices today.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>• AF80 184TB used — $79,500 or best offer (eBay, Core 4 Solutions).</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>• AF40 46TB (24×1.92TB SSD) new — $19,995 (eBay); used scaled to ~55–65% of new.</t>
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>PORTFOLIO SUMMARY (USD)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• AF40/60/80 92TB flash field-upgrade refurb — ~€53,550 (it-market.com) — corroborates AF-series SSD $/TB.</t>
+          <t>• Retail resale (reference) ......... ~$283,825 point</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>• Reseller-direct net offer ......... see Sheet 1 totals (≈ $139K point; ~$117K–$162K range)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>SOURCE LINKS</t>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>• Approx. haircut vs retail ......... ~50% (reseller margin) + minor data-wipe fee</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Enterasource — enterasource.com/storage/hpe-nimble</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ALTA Technologies — altatechnologies.com/collections/hpe-nimble-storage</t>
+          <t>MARKET ANCHORS (retail resale)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Spectra — spectra.com/hp/used-systems/83/Used-HP-Nimble-Storage.htm</t>
+          <t>• HF40 126TB HDD + 11.52TB SSD refurb — $16,875 (Enterasource) — exact match to array #1.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>eBay HF60 210TB — ebay.com/itm/176841322075</t>
+          <t>• HF60 210TB HDD + 23.04TB cache used — $23,995 (eBay).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>eBay AF60 184TB — ebay.com/itm/326495257900</t>
+          <t>• AF60 184TB (48×3.84TB SSD) used — $34,950 (eBay) — matches arrays #3/#4.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>eBay AF80 184TB — ebay.com/itm/166495997287</t>
+          <t>• AF80 184TB used — $79,500 or best offer (eBay).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>eBay AF40 46TB — ebay.com/itm/155085093828</t>
+          <t>• AF40 46TB (24×1.92TB SSD) new — $19,995 (eBay); used ~55–65% of new.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>it-market AF40/60/80 flash upgrade — it-market.com/en/components/controller-cards/hpe/af40</t>
-        </is>
-      </c>
+      <c r="A26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>SOURCE LINKS</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>DISCLAIMER</t>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Enterasource — enterasource.com/storage/hpe-nimble</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Figures are good-faith estimates for planning only, not offers or appraisals. The used-storage market moves quickly;</t>
+          <t>ALTA Technologies — altatechnologies.com/collections/hpe-nimble-storage</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>confirm with a formal quote from a licensed reseller (Enterasource, ALTA, Spectra, etc.) before any transaction.</t>
+          <t>Spectra — spectra.com/hp/used-systems/83/Used-HP-Nimble-Storage.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>eBay HF60 210TB — ebay.com/itm/176841322075</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>eBay AF60 184TB — ebay.com/itm/326495257900</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>eBay AF80 184TB — ebay.com/itm/166495997287</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>eBay AF40 46TB — ebay.com/itm/155085093828</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>it-market AF40/60/80 flash upgrade — it-market.com/en/components/controller-cards/hpe/af40</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
+        <is>
+          <t>NEGOTIATION NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>• Get the data-wipe / Certificate of Destruction stated in writing as included at no charge — some resellers net it out of the offer (modeled here).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>• Ask the reseller to itemize wipe cost vs. hardware value so you can see the true hardware offer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>• Est. drive counts are approximate (drive sizes not in the source inventory); wipe fee is immaterial to the total either way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>• If security policy ever requires PHYSICAL media destruction (shred), arrays sell diskless and offers drop sharply — not the case here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="inlineStr">
+        <is>
+          <t>DISCLAIMER</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Good-faith planning estimates only — not offers or formal appraisals. Confirm with written quotes from licensed resellers before transacting.</t>
         </is>
       </c>
     </row>

</xml_diff>